<commit_message>
fix that it will not contains a number to their name
</commit_message>
<xml_diff>
--- a/project/students.xlsx
+++ b/project/students.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Students" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Students'!$A$1:$L$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Students'!$A$1:$L$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -57,10 +57,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -427,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -506,8 +509,70 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>2025-00553-MN-2</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Dela Cruz, Princess Mae, M.</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Bachelor of Secondary Education Major in Social Studies</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>3rd year</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>09291234579</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Bacoor, Cavite</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Aileen Ramos</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Father</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>09407654333</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L1"/>
+  <autoFilter ref="A1:L2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
restricted no random letter for the name
</commit_message>
<xml_diff>
--- a/project/students.xlsx
+++ b/project/students.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Students" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Students'!$A$1:$L$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Students'!$A$1:$L$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -512,12 +512,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2025-00553-MN-2</t>
+          <t>2025-00543-MN-2</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Dela Cruz, Princess Mae, M.</t>
+          <t>Santos, Princess Mae</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -532,47 +532,295 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>09191234569</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Bacoor, Cavite</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Aileen Ramos</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Guardian</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>09307654323</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2025-00579-PS-8</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Garcia, Angelica Rose</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Diploma in Computer Engineering Technology</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>4th year</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>09551234605</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Dasmarinas, Cavite</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Nestor Dela Cruz</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Guardian</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>09667654359</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>2025-00548-MK-7</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Santos, Christian Paul, H.</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Bachelor of Science in Business Administration Major in Human Resource Management</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>3rd year</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>09241234574</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Taguig City</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Rosalinda Santos</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Mother</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>09357654328</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>2025-00590-TG-9</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Mendoza, Jerome Luis</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Diploma in Information Technology</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>5th year</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>09661234616</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Antipolo, Rizal</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Gloria Reyes</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Mother</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>09777654370</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>2025-00625-QC-4</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Bautista, Andrea Nicole, G.</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Bachelor of Science in Information Technology</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>5th year</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
           <t>22</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Female</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>09291234579</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Bacoor, Cavite</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>Aileen Ramos</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>09211234651</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Marikina City</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Jose Flores</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>Father</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>09407654333</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>09427654405</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L2"/>
+  <autoFilter ref="A1:L6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>